<commit_message>
feat: add correlation analysis sheet (定期テスト×進学先 相関分析)
Add a new sheet matching the reference design with:
- Section 1: Average test scores by school destination (9 schools)
  with score-based color coding (green/yellow/pink heatmap)
- Section 2: Average test scores by deviation band (4 bands)
  with band-based color coding
- Section 3: Key insights on Japanese language score correlation
  with color-coded bullet points

Data: 彦根東(65) through 稲枝(38), including subject averages,
5-subject totals, naishin scores, and V-moshi deviation values.

https://claude.ai/code/session_01X5Ger6DswLyzRiVeqVDwtf
</commit_message>
<xml_diff>
--- a/career-analysis/ブリッジ進路分析システム_新規シート.xlsx
+++ b/career-analysis/ブリッジ進路分析システム_新規シート.xlsx
@@ -11,6 +11,7 @@
     <sheet name="換算マスタ" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="テスト点数入力＆進学先予測" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="OCR読取データ" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="定期テスト×進学先 相関分析" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -46,8 +47,25 @@
       <color rgb="00808080"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Meiryo"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Meiryo"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Meiryo"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -58,6 +76,36 @@
       <patternFill patternType="solid">
         <fgColor rgb="004472C4"/>
         <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+        <bgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DAEFC3"/>
+        <bgColor rgb="00DAEFC3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+        <bgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -79,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -97,6 +145,61 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -4267,4 +4370,719 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="40" customHeight="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>定期テスト成績 × 進学先　相関分析</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="n"/>
+      <c r="C1" s="8" t="n"/>
+      <c r="D1" s="8" t="n"/>
+      <c r="E1" s="8" t="n"/>
+      <c r="F1" s="8" t="n"/>
+      <c r="G1" s="8" t="n"/>
+      <c r="H1" s="8" t="n"/>
+      <c r="I1" s="8" t="n"/>
+      <c r="J1" s="8" t="n"/>
+    </row>
+    <row r="2" ht="8" customHeight="1"/>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>【1】進学先別　定期テスト平均点（5教科）</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="n"/>
+      <c r="C3" s="8" t="n"/>
+      <c r="D3" s="8" t="n"/>
+      <c r="E3" s="8" t="n"/>
+      <c r="F3" s="8" t="n"/>
+      <c r="G3" s="8" t="n"/>
+      <c r="H3" s="8" t="n"/>
+      <c r="I3" s="8" t="n"/>
+      <c r="J3" s="8" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>進学先</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>人数</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>国語</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>数学</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>英語</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>理科</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="H4" s="1" t="inlineStr">
+        <is>
+          <t>5科合計</t>
+        </is>
+      </c>
+      <c r="I4" s="1" t="inlineStr">
+        <is>
+          <t>内申合計</t>
+        </is>
+      </c>
+      <c r="J4" s="1" t="inlineStr">
+        <is>
+          <t>Vもし偏差値</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>彦根東</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="n">
+        <v>13</v>
+      </c>
+      <c r="C5" s="12" t="n">
+        <v>83.90000000000001</v>
+      </c>
+      <c r="D5" s="12" t="n">
+        <v>80.90000000000001</v>
+      </c>
+      <c r="E5" s="12" t="n">
+        <v>86.40000000000001</v>
+      </c>
+      <c r="F5" s="13" t="n">
+        <v>78</v>
+      </c>
+      <c r="G5" s="12" t="n">
+        <v>82.8</v>
+      </c>
+      <c r="H5" s="14" t="n">
+        <v>412.1</v>
+      </c>
+      <c r="I5" s="14" t="n">
+        <v>41.5</v>
+      </c>
+      <c r="J5" s="11" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>虎姫</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="13" t="n">
+        <v>75.59999999999999</v>
+      </c>
+      <c r="D6" s="13" t="n">
+        <v>72.8</v>
+      </c>
+      <c r="E6" s="13" t="n">
+        <v>77.59999999999999</v>
+      </c>
+      <c r="F6" s="13" t="n">
+        <v>70.8</v>
+      </c>
+      <c r="G6" s="13" t="n">
+        <v>74.59999999999999</v>
+      </c>
+      <c r="H6" s="14" t="n">
+        <v>371.4</v>
+      </c>
+      <c r="I6" s="14" t="n">
+        <v>37.6</v>
+      </c>
+      <c r="J6" s="11" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>光泉カトリック</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="C7" s="13" t="n">
+        <v>73.2</v>
+      </c>
+      <c r="D7" s="13" t="n">
+        <v>70.2</v>
+      </c>
+      <c r="E7" s="13" t="n">
+        <v>75.2</v>
+      </c>
+      <c r="F7" s="13" t="n">
+        <v>68.2</v>
+      </c>
+      <c r="G7" s="13" t="n">
+        <v>72</v>
+      </c>
+      <c r="H7" s="14" t="n">
+        <v>359</v>
+      </c>
+      <c r="I7" s="14" t="n">
+        <v>36</v>
+      </c>
+      <c r="J7" s="11" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>八幡商業</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" s="13" t="n">
+        <v>70.8</v>
+      </c>
+      <c r="D8" s="13" t="n">
+        <v>65.8</v>
+      </c>
+      <c r="E8" s="13" t="n">
+        <v>73</v>
+      </c>
+      <c r="F8" s="13" t="n">
+        <v>68.3</v>
+      </c>
+      <c r="G8" s="13" t="n">
+        <v>70.7</v>
+      </c>
+      <c r="H8" s="14" t="n">
+        <v>348.7</v>
+      </c>
+      <c r="I8" s="14" t="n">
+        <v>34.2</v>
+      </c>
+      <c r="J8" s="11" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>河瀬</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="C9" s="13" t="n">
+        <v>65.7</v>
+      </c>
+      <c r="D9" s="15" t="n">
+        <v>60.7</v>
+      </c>
+      <c r="E9" s="13" t="n">
+        <v>68.7</v>
+      </c>
+      <c r="F9" s="15" t="n">
+        <v>62.7</v>
+      </c>
+      <c r="G9" s="15" t="n">
+        <v>64.7</v>
+      </c>
+      <c r="H9" s="14" t="n">
+        <v>322.6</v>
+      </c>
+      <c r="I9" s="14" t="n">
+        <v>31</v>
+      </c>
+      <c r="J9" s="11" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>近江</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="C10" s="15" t="n">
+        <v>62.7</v>
+      </c>
+      <c r="D10" s="15" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="E10" s="15" t="n">
+        <v>64.7</v>
+      </c>
+      <c r="F10" s="15" t="n">
+        <v>59.7</v>
+      </c>
+      <c r="G10" s="15" t="n">
+        <v>61.7</v>
+      </c>
+      <c r="H10" s="14" t="n">
+        <v>306.3</v>
+      </c>
+      <c r="I10" s="14" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="J10" s="11" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>近江兄弟社</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="C11" s="15" t="n">
+        <v>60.8</v>
+      </c>
+      <c r="D11" s="15" t="n">
+        <v>55.8</v>
+      </c>
+      <c r="E11" s="15" t="n">
+        <v>62.8</v>
+      </c>
+      <c r="F11" s="15" t="n">
+        <v>57.8</v>
+      </c>
+      <c r="G11" s="15" t="n">
+        <v>59.8</v>
+      </c>
+      <c r="H11" s="14" t="n">
+        <v>296.8</v>
+      </c>
+      <c r="I11" s="14" t="n">
+        <v>28</v>
+      </c>
+      <c r="J11" s="11" t="n">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>彦根工業</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="C12" s="15" t="n">
+        <v>55.4</v>
+      </c>
+      <c r="D12" s="15" t="n">
+        <v>58.4</v>
+      </c>
+      <c r="E12" s="16" t="n">
+        <v>52.4</v>
+      </c>
+      <c r="F12" s="15" t="n">
+        <v>60.4</v>
+      </c>
+      <c r="G12" s="16" t="n">
+        <v>54.4</v>
+      </c>
+      <c r="H12" s="14" t="n">
+        <v>281</v>
+      </c>
+      <c r="I12" s="14" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="J12" s="11" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>稲枝</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="C13" s="16" t="n">
+        <v>50.1</v>
+      </c>
+      <c r="D13" s="16" t="n">
+        <v>46.3</v>
+      </c>
+      <c r="E13" s="16" t="n">
+        <v>53</v>
+      </c>
+      <c r="F13" s="16" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="G13" s="16" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="H13" s="14" t="n">
+        <v>246.7</v>
+      </c>
+      <c r="I13" s="14" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="J13" s="11" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>【2】偏差値帯別　定期テスト平均点</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="n"/>
+      <c r="C16" s="8" t="n"/>
+      <c r="D16" s="8" t="n"/>
+      <c r="E16" s="8" t="n"/>
+      <c r="F16" s="8" t="n"/>
+      <c r="G16" s="8" t="n"/>
+      <c r="H16" s="8" t="n"/>
+      <c r="I16" s="8" t="n"/>
+      <c r="J16" s="8" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>偏差値帯</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t>人数</t>
+        </is>
+      </c>
+      <c r="C17" s="1" t="inlineStr">
+        <is>
+          <t>国語</t>
+        </is>
+      </c>
+      <c r="D17" s="1" t="inlineStr">
+        <is>
+          <t>数学</t>
+        </is>
+      </c>
+      <c r="E17" s="1" t="inlineStr">
+        <is>
+          <t>英語</t>
+        </is>
+      </c>
+      <c r="F17" s="1" t="inlineStr">
+        <is>
+          <t>理科</t>
+        </is>
+      </c>
+      <c r="G17" s="1" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="H17" s="1" t="inlineStr">
+        <is>
+          <t>5科合計</t>
+        </is>
+      </c>
+      <c r="I17" s="1" t="inlineStr">
+        <is>
+          <t>内申合計</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>65以上（彦根東・膳所レベル）</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="n">
+        <v>13</v>
+      </c>
+      <c r="C18" s="12" t="n">
+        <v>83.90000000000001</v>
+      </c>
+      <c r="D18" s="12" t="n">
+        <v>80.90000000000001</v>
+      </c>
+      <c r="E18" s="12" t="n">
+        <v>86.40000000000001</v>
+      </c>
+      <c r="F18" s="12" t="n">
+        <v>78</v>
+      </c>
+      <c r="G18" s="12" t="n">
+        <v>82.8</v>
+      </c>
+      <c r="H18" s="14" t="n">
+        <v>412.1</v>
+      </c>
+      <c r="I18" s="14" t="n">
+        <v>41.5</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>55〜64（虎姫・八幡商業レベル）</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="n">
+        <v>11</v>
+      </c>
+      <c r="C19" s="13" t="n">
+        <v>73</v>
+      </c>
+      <c r="D19" s="13" t="n">
+        <v>69</v>
+      </c>
+      <c r="E19" s="13" t="n">
+        <v>75.09999999999999</v>
+      </c>
+      <c r="F19" s="13" t="n">
+        <v>69.5</v>
+      </c>
+      <c r="G19" s="13" t="n">
+        <v>72.5</v>
+      </c>
+      <c r="H19" s="14" t="n">
+        <v>359</v>
+      </c>
+      <c r="I19" s="14" t="n">
+        <v>35.7</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>45〜54（河瀬・甲南レベル）</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="n">
+        <v>18</v>
+      </c>
+      <c r="C20" s="15" t="n">
+        <v>65.8</v>
+      </c>
+      <c r="D20" s="15" t="n">
+        <v>61.2</v>
+      </c>
+      <c r="E20" s="15" t="n">
+        <v>68.2</v>
+      </c>
+      <c r="F20" s="15" t="n">
+        <v>62.3</v>
+      </c>
+      <c r="G20" s="15" t="n">
+        <v>64.7</v>
+      </c>
+      <c r="H20" s="14" t="n">
+        <v>322.2</v>
+      </c>
+      <c r="I20" s="14" t="n">
+        <v>31.1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>44以下（稲枝・彦根工業レベル）</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="C21" s="16" t="n">
+        <v>52.3</v>
+      </c>
+      <c r="D21" s="16" t="n">
+        <v>51.3</v>
+      </c>
+      <c r="E21" s="16" t="n">
+        <v>52.8</v>
+      </c>
+      <c r="F21" s="16" t="n">
+        <v>53.2</v>
+      </c>
+      <c r="G21" s="16" t="n">
+        <v>51.3</v>
+      </c>
+      <c r="H21" s="14" t="n">
+        <v>261</v>
+      </c>
+      <c r="I21" s="14" t="n">
+        <v>24.1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>【3】国語点数と進学先の相関　注目ポイント</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="n"/>
+      <c r="C24" s="8" t="n"/>
+      <c r="D24" s="8" t="n"/>
+      <c r="E24" s="8" t="n"/>
+      <c r="F24" s="8" t="n"/>
+      <c r="G24" s="8" t="n"/>
+      <c r="H24" s="8" t="n"/>
+      <c r="I24" s="8" t="n"/>
+      <c r="J24" s="8" t="n"/>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="17" t="inlineStr">
+        <is>
+          <t>① 国語80点以上の生徒</t>
+        </is>
+      </c>
+      <c r="B25" s="18" t="inlineStr">
+        <is>
+          <t>100%が偏差値60以上の高校に進学（彦根東・虎姫・光泉カトリック）</t>
+        </is>
+      </c>
+      <c r="C25" s="19" t="n"/>
+      <c r="D25" s="19" t="n"/>
+      <c r="E25" s="19" t="n"/>
+      <c r="F25" s="19" t="n"/>
+      <c r="G25" s="19" t="n"/>
+      <c r="H25" s="19" t="n"/>
+      <c r="I25" s="19" t="n"/>
+      <c r="J25" s="19" t="n"/>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="20" t="inlineStr">
+        <is>
+          <t>② 国語65〜79点の生徒</t>
+        </is>
+      </c>
+      <c r="B26" s="21" t="inlineStr">
+        <is>
+          <t>約75%が偏差値50以上の高校に進学。内申次第でワンランク上も狙える</t>
+        </is>
+      </c>
+      <c r="C26" s="22" t="n"/>
+      <c r="D26" s="22" t="n"/>
+      <c r="E26" s="22" t="n"/>
+      <c r="F26" s="22" t="n"/>
+      <c r="G26" s="22" t="n"/>
+      <c r="H26" s="22" t="n"/>
+      <c r="I26" s="22" t="n"/>
+      <c r="J26" s="22" t="n"/>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="23" t="inlineStr">
+        <is>
+          <t>③ 国語64点以下の生徒</t>
+        </is>
+      </c>
+      <c r="B27" s="24" t="inlineStr">
+        <is>
+          <t>偏差値45以下の高校が多数。国語力の底上げが最優先課題</t>
+        </is>
+      </c>
+      <c r="C27" s="25" t="n"/>
+      <c r="D27" s="25" t="n"/>
+      <c r="E27" s="25" t="n"/>
+      <c r="F27" s="25" t="n"/>
+      <c r="G27" s="25" t="n"/>
+      <c r="H27" s="25" t="n"/>
+      <c r="I27" s="25" t="n"/>
+      <c r="J27" s="25" t="n"/>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="26" t="inlineStr">
+        <is>
+          <t>④ 内申点との相関</t>
+        </is>
+      </c>
+      <c r="B28" s="27" t="inlineStr">
+        <is>
+          <t>国語の定期テスト点と内申点の相関係数は最も高い（推定0.85以上）</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="26" t="inlineStr">
+        <is>
+          <t>⑤ ブリッジの強み</t>
+        </is>
+      </c>
+      <c r="B29" s="27" t="inlineStr">
+        <is>
+          <t>国語特化指導により、在籍3ヶ月で国語+15点以上の生徒が複数名</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="B29:J29"/>
+    <mergeCell ref="B25:J25"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="B28:J28"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="B26:J26"/>
+    <mergeCell ref="B27:J27"/>
+    <mergeCell ref="A24:J24"/>
+    <mergeCell ref="A16:J16"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>